<commit_message>
Fase 1: Modo Copiloto, Editor de Prompt Web y Variables Dinamicas
</commit_message>
<xml_diff>
--- a/empresas.xlsx
+++ b/empresas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\David Capera\Desktop\bot-zenix\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD732878-4311-418C-869F-AD9A081C1129}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{786F2C0F-3274-46A1-A70A-65836182E35E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,24 +25,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>Nombre</t>
-  </si>
-  <si>
-    <t>Correo</t>
   </si>
   <si>
     <t>Contacto</t>
   </si>
   <si>
-    <t>Estado</t>
+    <t>Laura Sofia Hernandez</t>
   </si>
   <si>
-    <t>Sofiaoma25@gmail.com</t>
-  </si>
-  <si>
-    <t>Laura Sofia Hernandez</t>
+    <t>Negocio Ejemplo</t>
   </si>
 </sst>
 </file>
@@ -394,38 +388,40 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="19.125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="B2">
+        <v>3173058198</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2">
-        <v>3173058198</v>
+      <c r="B3">
+        <v>3001234567</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:D1 A2:C2" numberStoredAsText="1"/>
+    <ignoredError sqref="A1 A2 B1 B2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix version cache y userAgent para evitar bloqueo en Sincronizando
</commit_message>
<xml_diff>
--- a/empresas.xlsx
+++ b/empresas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\David Capera\Desktop\bot-zenix\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{786F2C0F-3274-46A1-A70A-65836182E35E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F6A3554-A335-4040-9D20-A66FF4B2EC05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>Nombre</t>
   </si>
@@ -34,9 +34,6 @@
   </si>
   <si>
     <t>Laura Sofia Hernandez</t>
-  </si>
-  <si>
-    <t>Negocio Ejemplo</t>
   </si>
 </sst>
 </file>
@@ -388,7 +385,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.125" bestFit="1" customWidth="1"/>
@@ -410,14 +407,6 @@
         <v>3173058198</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3">
-        <v>3001234567</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>

</xml_diff>